<commit_message>
notas projetos... junho corrigidas, okk
</commit_message>
<xml_diff>
--- a/05 Others/2026.1 Avaliação Projetos/Turma Introdução a Programação - WYD6376 Turma 3001 PRESENCIAL Wyden UniRuy 2026_1.xlsx
+++ b/05 Others/2026.1 Avaliação Projetos/Turma Introdução a Programação - WYD6376 Turma 3001 PRESENCIAL Wyden UniRuy 2026_1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YduqsArea1\Avaliações Yduqs 2022_2 BDQ 2023_1 2024_2\2026.1 Avaliação Projetos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39064938-0D19-43F5-8659-0E4FFAAD9ABD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE98E9F6-DB88-44D8-84EE-C7524534E4B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{DD6ED3E7-57DF-4A52-9E4C-63B0F7661B3D}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="42">
   <si>
     <t>ALUNO</t>
   </si>
@@ -96,9 +96,6 @@
   </si>
   <si>
     <t>AVS</t>
-  </si>
-  <si>
-    <t>SIM</t>
   </si>
   <si>
     <t>TRAB</t>
@@ -159,14 +156,20 @@
     <t>https://github.com/MairoCruz/Projeto</t>
   </si>
   <si>
-    <t>atrasado</t>
+    <t>SIM1</t>
+  </si>
+  <si>
+    <t>SIM2</t>
+  </si>
+  <si>
+    <t>atrasado; AV foi considerado o projeto app nota 1,6. Feita a conversão de peso para a AV 2 E PROJ 8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -197,6 +200,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -415,7 +426,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -476,6 +487,10 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -816,9 +831,9 @@
   <sheetFormatPr defaultColWidth="59.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="59" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.140625" customWidth="1"/>
     <col min="3" max="3" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="7.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="5.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="24.85546875" bestFit="1" customWidth="1"/>
@@ -835,30 +850,30 @@
         <v>19</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
         <v>21</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="15" t="s">
-        <v>4</v>
+      <c r="B2" s="15">
+        <v>6.4</v>
       </c>
       <c r="C2" s="15" t="s">
         <v>4</v>
@@ -874,18 +889,18 @@
       </c>
       <c r="G2" s="15"/>
       <c r="H2" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
+      <c r="B3" s="1">
+        <v>8</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>4</v>
@@ -901,18 +916,18 @@
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>4</v>
+      <c r="B4" s="1">
+        <v>7.2</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>4</v>
@@ -928,18 +943,18 @@
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I4">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" s="12" t="s">
         <v>4</v>
@@ -955,18 +970,18 @@
       </c>
       <c r="G5" s="12"/>
       <c r="H5" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I5" s="20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>4</v>
+      <c r="B6" s="1">
+        <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>4</v>
@@ -982,18 +997,18 @@
       </c>
       <c r="G6" s="1"/>
       <c r="H6" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>4</v>
+      <c r="B7" s="12">
+        <v>7.2</v>
       </c>
       <c r="C7" s="12" t="s">
         <v>4</v>
@@ -1009,18 +1024,18 @@
       </c>
       <c r="G7" s="12"/>
       <c r="H7" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="1" t="s">
-        <v>4</v>
+      <c r="B8" s="1">
+        <v>8</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>4</v>
@@ -1036,18 +1051,18 @@
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="1" t="s">
-        <v>4</v>
+      <c r="B9" s="1">
+        <v>8</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>4</v>
@@ -1063,18 +1078,18 @@
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="63" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>4</v>
+      <c r="B10" s="12">
+        <v>8</v>
       </c>
       <c r="C10" s="12" t="s">
         <v>4</v>
@@ -1090,10 +1105,10 @@
       </c>
       <c r="G10" s="12"/>
       <c r="H10" s="13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:9" ht="15.75" x14ac:dyDescent="0.25">
@@ -1101,7 +1116,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C11" s="12" t="s">
         <v>4</v>
@@ -1117,15 +1132,15 @@
       </c>
       <c r="G11" s="12"/>
       <c r="H11" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="1" t="s">
-        <v>4</v>
+      <c r="B12" s="1">
+        <v>4.4000000000000004</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>4</v>
@@ -1137,22 +1152,22 @@
         <v>0.2</v>
       </c>
       <c r="F12" s="1">
-        <v>1.6</v>
+        <v>2</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="I12" t="s">
-        <v>40</v>
+        <v>38</v>
+      </c>
+      <c r="I12" s="21" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="1" t="s">
-        <v>4</v>
+      <c r="B13" s="1">
+        <v>6.4</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>4</v>
@@ -1168,15 +1183,15 @@
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:9" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B14" s="6" t="s">
-        <v>4</v>
+      <c r="B14" s="6">
+        <v>8</v>
       </c>
       <c r="C14" s="6" t="s">
         <v>4</v>
@@ -1192,10 +1207,10 @@
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I14" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>